<commit_message>
Scraper run: 2026-09-26 05:54 UTC
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$W$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$W$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,28 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00374151"/>
       <sz val="10"/>
     </font>
     <font>
@@ -49,7 +71,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +81,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E2433"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,14 +120,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -606,8 +656,1754 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>20260563011</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Superior Court</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>2801 N. Litchfield Rd., #75</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Goodyear</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>85395</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr"/>
+      <c r="T2" s="3" t="inlineStr"/>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>State Tax Lien</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>20260562756</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr"/>
+      <c r="O3" s="6" t="inlineStr"/>
+      <c r="P3" s="6" t="inlineStr"/>
+      <c r="Q3" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R3" s="6" t="inlineStr"/>
+      <c r="S3" s="6" t="inlineStr"/>
+      <c r="T3" s="6" t="inlineStr"/>
+      <c r="U3" s="6" t="inlineStr">
+        <is>
+          <t>Gov/Tax lien; New this week</t>
+        </is>
+      </c>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W3" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>20260561372</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr"/>
+      <c r="O4" s="6" t="inlineStr"/>
+      <c r="P4" s="6" t="inlineStr"/>
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R4" s="6" t="inlineStr"/>
+      <c r="S4" s="6" t="inlineStr"/>
+      <c r="T4" s="6" t="inlineStr"/>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W4" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>20260561373</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr"/>
+      <c r="O5" s="6" t="inlineStr"/>
+      <c r="P5" s="6" t="inlineStr"/>
+      <c r="Q5" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R5" s="6" t="inlineStr"/>
+      <c r="S5" s="6" t="inlineStr"/>
+      <c r="T5" s="6" t="inlineStr"/>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W5" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>20260561378</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Superior Court</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr"/>
+      <c r="O6" s="6" t="inlineStr"/>
+      <c r="P6" s="6" t="inlineStr"/>
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R6" s="6" t="inlineStr"/>
+      <c r="S6" s="6" t="inlineStr"/>
+      <c r="T6" s="6" t="inlineStr"/>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W6" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>20260562199</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W7" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>20260562308</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr"/>
+      <c r="O8" s="6" t="inlineStr"/>
+      <c r="P8" s="6" t="inlineStr"/>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R8" s="6" t="inlineStr"/>
+      <c r="S8" s="6" t="inlineStr"/>
+      <c r="T8" s="6" t="inlineStr"/>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V8" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W8" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>20260562328</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="inlineStr"/>
+      <c r="U9" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W9" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>20260562363</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Superior Court</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr"/>
+      <c r="O10" s="6" t="inlineStr"/>
+      <c r="P10" s="6" t="inlineStr"/>
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R10" s="6" t="inlineStr"/>
+      <c r="S10" s="6" t="inlineStr"/>
+      <c r="T10" s="6" t="inlineStr"/>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W10" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>20260562364</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr"/>
+      <c r="O11" s="6" t="inlineStr"/>
+      <c r="P11" s="6" t="inlineStr"/>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr"/>
+      <c r="S11" s="6" t="inlineStr"/>
+      <c r="T11" s="6" t="inlineStr"/>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W11" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>20260562428</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr"/>
+      <c r="O12" s="6" t="inlineStr"/>
+      <c r="P12" s="6" t="inlineStr"/>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R12" s="6" t="inlineStr"/>
+      <c r="S12" s="6" t="inlineStr"/>
+      <c r="T12" s="6" t="inlineStr"/>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W12" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>20260562445</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="inlineStr"/>
+      <c r="O13" s="6" t="inlineStr"/>
+      <c r="P13" s="6" t="inlineStr"/>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R13" s="6" t="inlineStr"/>
+      <c r="S13" s="6" t="inlineStr"/>
+      <c r="T13" s="6" t="inlineStr"/>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W13" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>20260562536</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr"/>
+      <c r="O14" s="6" t="inlineStr"/>
+      <c r="P14" s="6" t="inlineStr"/>
+      <c r="Q14" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R14" s="6" t="inlineStr"/>
+      <c r="S14" s="6" t="inlineStr"/>
+      <c r="T14" s="6" t="inlineStr"/>
+      <c r="U14" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W14" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>20260562810</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Superior Court |</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr"/>
+      <c r="O15" s="6" t="inlineStr"/>
+      <c r="P15" s="6" t="inlineStr"/>
+      <c r="Q15" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R15" s="6" t="inlineStr"/>
+      <c r="S15" s="6" t="inlineStr"/>
+      <c r="T15" s="6" t="inlineStr"/>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W15" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>20260563165</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Superior Court</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr"/>
+      <c r="O16" s="6" t="inlineStr"/>
+      <c r="P16" s="6" t="inlineStr"/>
+      <c r="Q16" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R16" s="6" t="inlineStr"/>
+      <c r="S16" s="6" t="inlineStr"/>
+      <c r="T16" s="6" t="inlineStr"/>
+      <c r="U16" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W16" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>20260563293</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>Superior Court in case no. CV2024-015783 on February 24</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="inlineStr"/>
+      <c r="U17" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W17" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>20260563301</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr"/>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr"/>
+      <c r="O18" s="6" t="inlineStr"/>
+      <c r="P18" s="6" t="inlineStr"/>
+      <c r="Q18" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R18" s="6" t="inlineStr"/>
+      <c r="S18" s="6" t="inlineStr"/>
+      <c r="T18" s="6" t="inlineStr"/>
+      <c r="U18" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W18" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>20260563302</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr"/>
+      <c r="O19" s="6" t="inlineStr"/>
+      <c r="P19" s="6" t="inlineStr"/>
+      <c r="Q19" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R19" s="6" t="inlineStr"/>
+      <c r="S19" s="6" t="inlineStr"/>
+      <c r="T19" s="6" t="inlineStr"/>
+      <c r="U19" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V19" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W19" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>20260563510</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr"/>
+      <c r="O20" s="6" t="inlineStr"/>
+      <c r="P20" s="6" t="inlineStr"/>
+      <c r="Q20" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R20" s="6" t="inlineStr"/>
+      <c r="S20" s="6" t="inlineStr"/>
+      <c r="T20" s="6" t="inlineStr"/>
+      <c r="U20" s="6" t="inlineStr">
+        <is>
+          <t>Judgment lien; New this week</t>
+        </is>
+      </c>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W20" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>20260562677</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="inlineStr"/>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr"/>
+      <c r="O21" s="6" t="inlineStr"/>
+      <c r="P21" s="6" t="inlineStr"/>
+      <c r="Q21" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R21" s="6" t="inlineStr"/>
+      <c r="S21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="inlineStr"/>
+      <c r="U21" s="6" t="inlineStr">
+        <is>
+          <t>Probate / estate; New this week</t>
+        </is>
+      </c>
+      <c r="V21" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W21" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>20260562679</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA |</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N22" s="6" t="inlineStr"/>
+      <c r="O22" s="6" t="inlineStr"/>
+      <c r="P22" s="6" t="inlineStr"/>
+      <c r="Q22" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R22" s="6" t="inlineStr"/>
+      <c r="S22" s="6" t="inlineStr"/>
+      <c r="T22" s="6" t="inlineStr"/>
+      <c r="U22" s="6" t="inlineStr">
+        <is>
+          <t>Probate / estate; New this week</t>
+        </is>
+      </c>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W22" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>20260562681</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr"/>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr"/>
+      <c r="O23" s="6" t="inlineStr"/>
+      <c r="P23" s="6" t="inlineStr"/>
+      <c r="Q23" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="inlineStr"/>
+      <c r="S23" s="6" t="inlineStr"/>
+      <c r="T23" s="6" t="inlineStr"/>
+      <c r="U23" s="6" t="inlineStr">
+        <is>
+          <t>Probate / estate; New this week</t>
+        </is>
+      </c>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W23" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>20260562683</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr"/>
+      <c r="O24" s="6" t="inlineStr"/>
+      <c r="P24" s="6" t="inlineStr"/>
+      <c r="Q24" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R24" s="6" t="inlineStr"/>
+      <c r="S24" s="6" t="inlineStr"/>
+      <c r="T24" s="6" t="inlineStr"/>
+      <c r="U24" s="6" t="inlineStr">
+        <is>
+          <t>Probate / estate; New this week</t>
+        </is>
+      </c>
+      <c r="V24" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W24" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>20260562685</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N25" s="6" t="inlineStr"/>
+      <c r="O25" s="6" t="inlineStr"/>
+      <c r="P25" s="6" t="inlineStr"/>
+      <c r="Q25" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R25" s="6" t="inlineStr"/>
+      <c r="S25" s="6" t="inlineStr"/>
+      <c r="T25" s="6" t="inlineStr"/>
+      <c r="U25" s="6" t="inlineStr">
+        <is>
+          <t>Probate / estate; New this week</t>
+        </is>
+      </c>
+      <c r="V25" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W25" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>20260562688</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N26" s="6" t="inlineStr"/>
+      <c r="O26" s="6" t="inlineStr"/>
+      <c r="P26" s="6" t="inlineStr"/>
+      <c r="Q26" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R26" s="6" t="inlineStr"/>
+      <c r="S26" s="6" t="inlineStr">
+        <is>
+          <t>102-23-015</t>
+        </is>
+      </c>
+      <c r="T26" s="6" t="inlineStr"/>
+      <c r="U26" s="6" t="inlineStr">
+        <is>
+          <t>Probate / estate; New this week</t>
+        </is>
+      </c>
+      <c r="V26" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W26" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>20260563023</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>SUPERIOR COURT OF THE STATE OF ARIZONA</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr"/>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N27" s="6" t="inlineStr"/>
+      <c r="O27" s="6" t="inlineStr"/>
+      <c r="P27" s="6" t="inlineStr"/>
+      <c r="Q27" s="6" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R27" s="6" t="inlineStr"/>
+      <c r="S27" s="6" t="inlineStr"/>
+      <c r="T27" s="6" t="inlineStr"/>
+      <c r="U27" s="6" t="inlineStr">
+        <is>
+          <t>Probate / estate; New this week</t>
+        </is>
+      </c>
+      <c r="V27" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W27" s="7" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
+  <autoFilter ref="A1:W27"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W27" r:id="rId26"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -618,7 +2414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -626,7 +2422,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Maricopa County Motivated Seller Leads</t>
         </is>
@@ -635,88 +2431,118 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run: 2026-09-25 05:52</t>
+          <t>Run: 2026-09-26 05:54</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr"/>
-      <c r="B3" s="3" t="inlineStr"/>
+      <c r="A3" s="9" t="inlineStr"/>
+      <c r="B3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Total Leads</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="9" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>With Property Address</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>With Mailing Address</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>With Property Address</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>PDF Parsed</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Score 70+ (Hot)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>With Mailing Address</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>PDF Parsed</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Score 70+ (Hot)</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Score 50-69 (Warm)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>0</v>
+      <c r="B9" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="A10" s="9" t="inlineStr"/>
+      <c r="B10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>By Category</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Probate Document</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>State Tax Lien</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Scraper run: 2026-10-03 06:08 UTC
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$W$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$W$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,22 +37,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00374151"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="002563EB"/>
-      <sz val="9"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
@@ -65,7 +49,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -75,11 +59,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E2433"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,23 +88,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -636,418 +606,8 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Probate Document</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>PD</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>20260574924</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>SUPERIOR COURT OF ARIZONA</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr"/>
-      <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr"/>
-      <c r="S2" s="3" t="inlineStr"/>
-      <c r="T2" s="3" t="inlineStr"/>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>Probate / estate; New this week</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W2" s="4" t="inlineStr">
-        <is>
-          <t>View ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Probate Document</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>20260573920</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>SUPERIOR COURT OF ARIZONA</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr"/>
-      <c r="S3" s="3" t="inlineStr"/>
-      <c r="T3" s="3" t="inlineStr"/>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>Probate / estate; New this week</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W3" s="4" t="inlineStr">
-        <is>
-          <t>View ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Probate Document</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>20260574216</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>SUPERIOR COURT :</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="3" t="inlineStr"/>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="inlineStr"/>
-      <c r="S4" s="3" t="inlineStr"/>
-      <c r="T4" s="3" t="inlineStr"/>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>Probate / estate; New this week</t>
-        </is>
-      </c>
-      <c r="V4" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W4" s="4" t="inlineStr">
-        <is>
-          <t>View ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Probate Document</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>20260574640</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>SUPERIOR COURT</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr"/>
-      <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="3" t="inlineStr"/>
-      <c r="Q5" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="inlineStr"/>
-      <c r="S5" s="3" t="inlineStr"/>
-      <c r="T5" s="3" t="inlineStr"/>
-      <c r="U5" s="3" t="inlineStr">
-        <is>
-          <t>Probate / estate; New this week</t>
-        </is>
-      </c>
-      <c r="V5" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W5" s="4" t="inlineStr">
-        <is>
-          <t>View ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Probate Document</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>20260574678</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>SUPERIOR COURT</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr"/>
-      <c r="O6" s="3" t="inlineStr"/>
-      <c r="P6" s="3" t="inlineStr"/>
-      <c r="Q6" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="R6" s="3" t="inlineStr"/>
-      <c r="S6" s="3" t="inlineStr"/>
-      <c r="T6" s="3" t="inlineStr"/>
-      <c r="U6" s="3" t="inlineStr">
-        <is>
-          <t>Probate / estate; New this week</t>
-        </is>
-      </c>
-      <c r="V6" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W6" s="4" t="inlineStr">
-        <is>
-          <t>View ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Probate Document</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>20260575012</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>SUPERIOR COURT</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr"/>
-      <c r="O7" s="3" t="inlineStr"/>
-      <c r="P7" s="3" t="inlineStr"/>
-      <c r="Q7" s="3" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="inlineStr"/>
-      <c r="S7" s="3" t="inlineStr"/>
-      <c r="T7" s="3" t="inlineStr"/>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>Probate / estate; New this week</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W7" s="4" t="inlineStr">
-        <is>
-          <t>View ↗</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W7"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" r:id="rId6"/>
-  </hyperlinks>
+  <autoFilter ref="A1:W1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1058,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1066,7 +626,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Maricopa County Motivated Seller Leads</t>
         </is>
@@ -1075,98 +635,88 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run: 2026-10-02 06:45</t>
+          <t>Run: 2026-10-03 06:08</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr"/>
-      <c r="B3" s="6" t="inlineStr"/>
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Total Leads</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
-        <v>6</v>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>With Property Address</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>With Mailing Address</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>PDF Parsed</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>6</v>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Score 70+ (Hot)</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Score 50-69 (Warm)</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr"/>
-      <c r="B10" s="6" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>By Category</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Probate Document</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Scraper run: 2026-10-07 06:57 UTC
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$W$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$W$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,22 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00374151"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
@@ -49,7 +65,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E2433"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,14 +109,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -606,8 +636,342 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Tax Deed</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>20260580703</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Superior Court of the State of</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr"/>
+      <c r="T2" s="3" t="inlineStr"/>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>Tax deed; New this week</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tax Deed</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>20260581668</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr"/>
+      <c r="S3" s="3" t="inlineStr"/>
+      <c r="T3" s="3" t="inlineStr"/>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>Tax deed; New this week</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W3" s="4" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Tax Deed</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>20260581686</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>VICKI L. LESCOE</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr"/>
+      <c r="S4" s="3" t="inlineStr"/>
+      <c r="T4" s="3" t="inlineStr"/>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>Tax deed; New this week</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Tax Deed</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>20260581770</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr"/>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>503-50-558</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr"/>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>Tax deed; New this week</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Tax Deed</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>20260581804</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr"/>
+      <c r="S6" s="3" t="inlineStr"/>
+      <c r="T6" s="3" t="inlineStr"/>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>Tax deed; New this week</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="inlineStr">
+        <is>
+          <t>View ↗</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
+  <autoFilter ref="A1:W6"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -618,7 +982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -626,7 +990,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Maricopa County Motivated Seller Leads</t>
         </is>
@@ -635,88 +999,98 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run: 2026-10-06 07:17</t>
+          <t>Run: 2026-10-07 06:57</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr"/>
-      <c r="B3" s="3" t="inlineStr"/>
+      <c r="A3" s="6" t="inlineStr"/>
+      <c r="B3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Total Leads</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>With Property Address</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>With Property Address</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>With Mailing Address</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>With Mailing Address</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>PDF Parsed</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Score 70+ (Hot)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>PDF Parsed</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Score 50-69 (Warm)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Score 70+ (Hot)</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Score 50-69 (Warm)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="A10" s="6" t="inlineStr"/>
+      <c r="B10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>By Category</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Tax Deed</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>